<commit_message>
update bom non-stocked components  change repo name  regenerate fabrications outputs
</commit_message>
<xml_diff>
--- a/Project Outputs for UltraZohm_Analog_ADS5272/BOM/BOM_UltraZohm_Analog_ADS5272_3v01.xlsx
+++ b/Project Outputs for UltraZohm_Analog_ADS5272/BOM/BOM_UltraZohm_Analog_ADS5272_3v01.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hm-kreppel\Documents\Altium Projects\ultrazohm_analog_ads5272_1vxx\Project Outputs for UltraZohm_Analog_ADS5272\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UltraZohm\UZ_A_ADS5272\Project Outputs for UltraZohm_Analog_ADS5272\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA073265-B7E8-4B9F-B90A-F3382FBC5970}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="11565"/>
+    <workbookView xWindow="2250" yWindow="1770" windowWidth="14670" windowHeight="8325" xr2:uid="{42211160-A3CD-495D-9319-87AC5872E5BB}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UltraZohm_Analog_ADS5272_3v" sheetId="1" r:id="rId1"/>
@@ -17,17 +18,26 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">BOM_UltraZohm_Analog_ADS5272_3v!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="287">
   <si>
     <t>Name</t>
   </si>
@@ -473,7 +483,7 @@
     <t>0</t>
   </si>
   <si>
-    <t>R14, R41, R48</t>
+    <t>R14, R29A, R29B, R30A, R30B, R41, R42A, R42B, R47A, R47B, R48</t>
   </si>
   <si>
     <t>RC0603JR-070RL</t>
@@ -488,7 +498,10 @@
     <t>R16</t>
   </si>
   <si>
-    <t>RC0603FR-074K7L</t>
+    <t>Vishay</t>
+  </si>
+  <si>
+    <t>CRCW04025R10JNEDC</t>
   </si>
   <si>
     <t>311-4.70KHRCT-ND</t>
@@ -839,10 +852,13 @@
     <t>SOT230P700X170-4N</t>
   </si>
   <si>
-    <t>TLV1117LV18DCYR</t>
-  </si>
-  <si>
-    <t>296-28777-1-ND</t>
+    <t>TLV1117LV18DCYT</t>
+  </si>
+  <si>
+    <t>Mouser</t>
+  </si>
+  <si>
+    <t>595-TLV1117LV18DCYT</t>
   </si>
   <si>
     <t>20MHz</t>
@@ -857,19 +873,37 @@
     <t>CRYSTALOSC</t>
   </si>
   <si>
-    <t>CTS-Frequency Controls</t>
-  </si>
-  <si>
-    <t>CB3LV-3I-20M000000</t>
-  </si>
-  <si>
-    <t>110-CB3LV-3I-20M000000CT-ND</t>
+    <t>CTS</t>
+  </si>
+  <si>
+    <t>CB3LV-3C-20M000000</t>
+  </si>
+  <si>
+    <t>110-CB3LV-3C-20M000000CT-ND</t>
+  </si>
+  <si>
+    <t>MPN</t>
+  </si>
+  <si>
+    <t>X3</t>
+  </si>
+  <si>
+    <t>2.54mm Double Row Terminal Assembly, Right-Angled</t>
+  </si>
+  <si>
+    <t>IPL1-102-01-L-D-K</t>
+  </si>
+  <si>
+    <t>Samtec</t>
+  </si>
+  <si>
+    <t>SAM10565-ND</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -934,7 +968,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -950,7 +984,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -966,7 +1000,7 @@
         <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
         <a:srgbClr val="ED7D31"/>
@@ -978,7 +1012,7 @@
         <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
         <a:srgbClr val="70AD47"/>
@@ -1025,6 +1059,23 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri" panose="020F0502020204030204"/>
@@ -1060,6 +1111,23 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
+        <a:font script="Armn" typeface="Arial"/>
+        <a:font script="Bugi" typeface="Leelawadee UI"/>
+        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
+        <a:font script="Java" typeface="Javanese Text"/>
+        <a:font script="Lisu" typeface="Segoe UI"/>
+        <a:font script="Mymr" typeface="Myanmar Text"/>
+        <a:font script="Nkoo" typeface="Ebrima"/>
+        <a:font script="Olck" typeface="Nirmala UI"/>
+        <a:font script="Osma" typeface="Ebrima"/>
+        <a:font script="Phag" typeface="Phagspa"/>
+        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
+        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
+        <a:font script="Syre" typeface="Estrangelo Edessa"/>
+        <a:font script="Sora" typeface="Nirmala UI"/>
+        <a:font script="Tale" typeface="Microsoft Tai Le"/>
+        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
+        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1211,25 +1279,25 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25604C2F-87A8-4494-B7F1-F0A4A6F7BFAE}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P49"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" customWidth="1"/>
-    <col min="2" max="2" width="17.7109375" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" customWidth="1"/>
-    <col min="4" max="4" width="12.85546875" customWidth="1"/>
-    <col min="5" max="8" width="16.7109375" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="11" width="16.7109375" customWidth="1"/>
-    <col min="12" max="12" width="12.42578125" customWidth="1"/>
-    <col min="13" max="13" width="15.85546875" customWidth="1"/>
-    <col min="14" max="14" width="16.7109375" customWidth="1"/>
-    <col min="15" max="15" width="10.7109375" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.5703125" customWidth="1"/>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="12.7109375" customWidth="1"/>
+    <col min="5" max="8" width="16.5703125" customWidth="1"/>
+    <col min="9" max="9" width="12.7109375" customWidth="1"/>
+    <col min="10" max="11" width="16.5703125" customWidth="1"/>
+    <col min="12" max="12" width="12.28515625" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" customWidth="1"/>
+    <col min="14" max="14" width="16.5703125" customWidth="1"/>
+    <col min="15" max="15" width="10.5703125" customWidth="1"/>
+    <col min="16" max="16" width="16.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
@@ -1282,7 +1350,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
@@ -1670,7 +1738,7 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>72</v>
       </c>
@@ -1938,7 +2006,7 @@
         <v>1.1200000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:16" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>102</v>
       </c>
@@ -2284,7 +2352,7 @@
         <v>1.44</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>147</v>
       </c>
@@ -2324,10 +2392,10 @@
         <v>1.7000000000000001E-2</v>
       </c>
       <c r="O24" s="4">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="P24" s="4">
-        <v>0.17</v>
+        <v>0.187</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
@@ -2355,16 +2423,16 @@
         <v>130</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="N25" s="4">
         <v>0.1</v>
@@ -2378,13 +2446,13 @@
     </row>
     <row r="26" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B26" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="C26" s="3" t="s">
         <v>156</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>155</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>107</v>
@@ -2404,13 +2472,13 @@
         <v>136</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="N26" s="4">
         <v>0.1</v>
@@ -2424,13 +2492,13 @@
     </row>
     <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="C27" s="3" t="s">
         <v>160</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>159</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>107</v>
@@ -2450,13 +2518,13 @@
         <v>136</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="N27" s="4">
         <v>0.17</v>
@@ -2473,32 +2541,32 @@
         <v>143</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>143</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L28" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M28" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N28" s="4">
         <v>0.60299999999999998</v>
@@ -2512,35 +2580,35 @@
     </row>
     <row r="29" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B29" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="C29" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="C29" s="3" t="s">
-        <v>169</v>
-      </c>
       <c r="D29" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="N29" s="4">
         <v>0.77</v>
@@ -2554,13 +2622,13 @@
     </row>
     <row r="30" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>174</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>173</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>107</v>
@@ -2580,13 +2648,13 @@
         <v>136</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="N30" s="4">
         <v>0.1</v>
@@ -2600,16 +2668,16 @@
     </row>
     <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B31" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C31" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="C31" s="3" t="s">
-        <v>177</v>
-      </c>
       <c r="D31" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E31" s="3" t="s">
         <v>19</v>
@@ -2623,16 +2691,16 @@
         <v>20</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="N31" s="4">
         <v>0.22</v>
@@ -2646,13 +2714,13 @@
     </row>
     <row r="32" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B32" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>184</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>183</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>107</v>
@@ -2661,7 +2729,7 @@
         <v>28</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
@@ -2669,16 +2737,16 @@
         <v>130</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="N32" s="4">
         <v>0.26</v>
@@ -2692,13 +2760,13 @@
     </row>
     <row r="33" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B33" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="C33" s="3" t="s">
         <v>190</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>189</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>107</v>
@@ -2707,7 +2775,7 @@
         <v>28</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
@@ -2715,16 +2783,16 @@
         <v>130</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="N33" s="4">
         <v>0.26</v>
@@ -2738,13 +2806,13 @@
     </row>
     <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>107</v>
@@ -2764,13 +2832,13 @@
         <v>136</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L34" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="N34" s="4">
         <v>0.1</v>
@@ -2784,13 +2852,13 @@
     </row>
     <row r="35" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B35" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>197</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>196</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>107</v>
@@ -2810,13 +2878,13 @@
         <v>136</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="L35" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="N35" s="4">
         <v>0.1</v>
@@ -2830,22 +2898,22 @@
     </row>
     <row r="36" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B36" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>201</v>
       </c>
-      <c r="C36" s="3" t="s">
-        <v>200</v>
-      </c>
       <c r="D36" s="3" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E36" s="3" t="s">
         <v>19</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -2853,16 +2921,16 @@
         <v>20</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K36" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L36" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M36" s="3" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="N36" s="4">
         <v>0.41</v>
@@ -2876,13 +2944,13 @@
     </row>
     <row r="37" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B37" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>206</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>205</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>107</v>
@@ -2902,13 +2970,13 @@
         <v>136</v>
       </c>
       <c r="K37" s="3" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="L37" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M37" s="3" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="N37" s="4">
         <v>0.1</v>
@@ -2922,10 +2990,10 @@
     </row>
     <row r="38" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="3" t="s">
@@ -2936,19 +3004,19 @@
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="3" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K38" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="L38" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M38" s="3" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="N38" s="4">
         <v>3.98</v>
@@ -2962,35 +3030,35 @@
     </row>
     <row r="39" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="3" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K39" s="3" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="L39" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M39" s="3" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="N39" s="4">
         <v>7.33</v>
@@ -3004,33 +3072,33 @@
     </row>
     <row r="40" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="3" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K40" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L40" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="N40" s="4">
         <v>3.83</v>
@@ -3044,10 +3112,10 @@
     </row>
     <row r="41" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="3" t="s">
@@ -3058,19 +3126,19 @@
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
       <c r="I41" s="3" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="L41" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="N41" s="4">
         <v>124.86</v>
@@ -3084,33 +3152,33 @@
     </row>
     <row r="42" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L42" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="N42" s="4">
         <v>0.32</v>
@@ -3124,33 +3192,33 @@
     </row>
     <row r="43" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="L43" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N43" s="4">
         <v>7</v>
@@ -3164,33 +3232,33 @@
     </row>
     <row r="44" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="3" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K44" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L44" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="N44" s="4">
         <v>0.53</v>
@@ -3204,33 +3272,33 @@
     </row>
     <row r="45" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="N45" s="4"/>
       <c r="O45" s="4">
@@ -3240,33 +3308,33 @@
     </row>
     <row r="46" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E46" s="4"/>
       <c r="F46" s="4"/>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
       <c r="I46" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K46" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="L46" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M46" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="N46" s="4">
         <v>2.4300000000000002</v>
@@ -3280,81 +3348,131 @@
     </row>
     <row r="47" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C47" s="4"/>
       <c r="D47" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
       <c r="I47" s="3" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K47" s="3" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L47" s="3" t="s">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="M47" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="N47" s="4"/>
+        <v>273</v>
+      </c>
+      <c r="N47" s="4">
+        <v>0.56000000000000005</v>
+      </c>
       <c r="O47" s="4">
         <v>1</v>
       </c>
-      <c r="P47" s="4"/>
+      <c r="P47" s="4">
+        <v>0.56000000000000005</v>
+      </c>
     </row>
     <row r="48" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="K48" s="3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="L48" s="3" t="s">
-        <v>258</v>
+        <v>23</v>
       </c>
       <c r="M48" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="N48" s="4"/>
+        <v>280</v>
+      </c>
+      <c r="N48" s="4">
+        <v>1.41</v>
+      </c>
       <c r="O48" s="4">
         <v>1</v>
       </c>
-      <c r="P48" s="4"/>
+      <c r="P48" s="4">
+        <v>1.41</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>283</v>
+      </c>
+      <c r="E49" s="4"/>
+      <c r="F49" s="4"/>
+      <c r="G49" s="4"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="K49" s="3" t="s">
+        <v>284</v>
+      </c>
+      <c r="L49" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M49" s="3" t="s">
+        <v>286</v>
+      </c>
+      <c r="N49" s="4">
+        <v>3.64</v>
+      </c>
+      <c r="O49" s="4">
+        <v>1</v>
+      </c>
+      <c r="P49" s="4">
+        <v>3.64</v>
+      </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="19" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="19" orientation="landscape" horizontalDpi="4294967292" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Regenerate Fabrication outputs for SMD assembly variant.
</commit_message>
<xml_diff>
--- a/Project Outputs for UltraZohm_Analog_ADS5272/BOM/BOM_UltraZohm_Analog_ADS5272_3v01.xlsx
+++ b/Project Outputs for UltraZohm_Analog_ADS5272/BOM/BOM_UltraZohm_Analog_ADS5272_3v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UltraZohm\UZ_A_ADS5272\Project Outputs for UltraZohm_Analog_ADS5272\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA073265-B7E8-4B9F-B90A-F3382FBC5970}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{870F30B5-A0FE-43EF-BC63-1830E0C34554}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2250" yWindow="1770" windowWidth="14670" windowHeight="8325" xr2:uid="{42211160-A3CD-495D-9319-87AC5872E5BB}"/>
+    <workbookView xWindow="2940" yWindow="2460" windowWidth="14670" windowHeight="8325" xr2:uid="{43EB9E44-8CEF-4548-86FA-A424F98C0A85}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UltraZohm_Analog_ADS5272_3v" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="262">
   <si>
     <t>Name</t>
   </si>
@@ -216,27 +216,6 @@
     <t>732-7766-1-ND</t>
   </si>
   <si>
-    <t>68µF</t>
-  </si>
-  <si>
-    <t>C60, C61</t>
-  </si>
-  <si>
-    <t>WCAP-ATG8 THT Aluminum Electrolytic Capacitors, D6.3mm x L11mm, 68uF, +/-20%, 35VDC</t>
-  </si>
-  <si>
-    <t>+/-20%</t>
-  </si>
-  <si>
-    <t>WCAP-ATG8_6.3x11</t>
-  </si>
-  <si>
-    <t>860010573006</t>
-  </si>
-  <si>
-    <t>732-8736-1-ND</t>
-  </si>
-  <si>
     <t>10µF</t>
   </si>
   <si>
@@ -345,94 +324,61 @@
     <t>732-4981-1-ND</t>
   </si>
   <si>
-    <t>RJHSE-5380-02</t>
-  </si>
-  <si>
-    <t>J1</t>
-  </si>
-  <si>
-    <t>Modular Jack WR-MJ, Tab Up, Shielded, Dual Port, Righ Angle, THT, 8P8C</t>
-  </si>
-  <si>
-    <t>Amphenol ICC</t>
-  </si>
-  <si>
-    <t>RJHSE-5380-02-ND</t>
+    <t>15mH</t>
+  </si>
+  <si>
+    <t>L2</t>
+  </si>
+  <si>
+    <t>SMT power Inductor, 15uH, 40m DRC</t>
+  </si>
+  <si>
+    <t>SMT_inductor_1050_Performance</t>
+  </si>
+  <si>
+    <t>48150SC</t>
+  </si>
+  <si>
+    <t>811-3837-1-ND</t>
+  </si>
+  <si>
+    <t>X95840_</t>
+  </si>
+  <si>
+    <t>POT1, POT2</t>
+  </si>
+  <si>
+    <t>Digital Trimmer</t>
+  </si>
+  <si>
+    <t>TSSO6X6-G20/D6.6</t>
+  </si>
+  <si>
+    <t>Intersil</t>
+  </si>
+  <si>
+    <t>X95840WV20IZ-2.7</t>
+  </si>
+  <si>
+    <t>X95840WV20IZ-2.7-ND</t>
+  </si>
+  <si>
+    <t>2.2k</t>
+  </si>
+  <si>
+    <t>R1, R2, R21, R22</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>JTAG CPLD</t>
-  </si>
-  <si>
-    <t>Header, 5-Pin, Dual row, Vertical</t>
-  </si>
-  <si>
-    <t>HEADER_JTAG - MAXII Horizontal</t>
-  </si>
-  <si>
-    <t>CNC Tech</t>
-  </si>
-  <si>
-    <t>3020-10-0200-00</t>
-  </si>
-  <si>
-    <t>1175-1615-ND</t>
-  </si>
-  <si>
-    <t>15mH</t>
-  </si>
-  <si>
-    <t>L2</t>
-  </si>
-  <si>
-    <t>SMT power Inductor, 15uH, 40m DRC</t>
-  </si>
-  <si>
-    <t>SMT_inductor_1050_Performance</t>
-  </si>
-  <si>
-    <t>48150SC</t>
-  </si>
-  <si>
-    <t>811-3837-1-ND</t>
-  </si>
-  <si>
-    <t>X95840_</t>
-  </si>
-  <si>
-    <t>POT1, POT2</t>
-  </si>
-  <si>
-    <t>Digital Trimmer</t>
-  </si>
-  <si>
-    <t>TSSO6X6-G20/D6.6</t>
-  </si>
-  <si>
-    <t>Intersil</t>
-  </si>
-  <si>
-    <t>X95840WV20IZ-2.7</t>
-  </si>
-  <si>
-    <t>X95840WV20IZ-2.7-ND</t>
-  </si>
-  <si>
-    <t>2.2k</t>
-  </si>
-  <si>
-    <t>R1, R2, R21, R22</t>
-  </si>
-  <si>
     <t>1%</t>
   </si>
   <si>
     <t>RES_0603</t>
   </si>
   <si>
-    <t>Yageo Phycomp</t>
+    <t>Yageo</t>
   </si>
   <si>
     <t>RC0603FR-072K2L</t>
@@ -447,9 +393,6 @@
     <t>R3, R20</t>
   </si>
   <si>
-    <t>Yageo</t>
-  </si>
-  <si>
     <t>RC0603JR-07220RL</t>
   </si>
   <si>
@@ -483,7 +426,7 @@
     <t>0</t>
   </si>
   <si>
-    <t>R14, R29A, R29B, R30A, R30B, R41, R42A, R42B, R47A, R47B, R48</t>
+    <t>R14, R41, R48</t>
   </si>
   <si>
     <t>RC0603JR-070RL</t>
@@ -880,24 +823,6 @@
   </si>
   <si>
     <t>110-CB3LV-3C-20M000000CT-ND</t>
-  </si>
-  <si>
-    <t>MPN</t>
-  </si>
-  <si>
-    <t>X3</t>
-  </si>
-  <si>
-    <t>2.54mm Double Row Terminal Assembly, Right-Angled</t>
-  </si>
-  <si>
-    <t>IPL1-102-01-L-D-K</t>
-  </si>
-  <si>
-    <t>Samtec</t>
-  </si>
-  <si>
-    <t>SAM10565-ND</t>
   </si>
 </sst>
 </file>
@@ -1279,11 +1204,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25604C2F-87A8-4494-B7F1-F0A4A6F7BFAE}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2344F444-6119-4E31-8C7D-B0DBEF4FE766}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -1642,7 +1567,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="135" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>59</v>
       </c>
@@ -1653,50 +1578,54 @@
         <v>59</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E8" s="4"/>
-      <c r="F8" s="3" t="s">
+      <c r="H8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="4"/>
-      <c r="I8" s="3" t="s">
+      <c r="K8" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="J8" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K8" s="3" t="s">
+      <c r="L8" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M8" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="L8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="N8" s="4">
-        <v>0.13</v>
+        <v>0.34</v>
       </c>
       <c r="O8" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P8" s="4">
-        <v>0.26</v>
+        <v>1.02</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>67</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>27</v>
@@ -1708,7 +1637,7 @@
         <v>29</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>31</v>
@@ -1717,36 +1646,36 @@
         <v>20</v>
       </c>
       <c r="J9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M9" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="K9" s="3" t="s">
+      <c r="N9" s="4">
+        <v>0.17</v>
+      </c>
+      <c r="O9" s="4">
+        <v>1</v>
+      </c>
+      <c r="P9" s="4">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="L9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="N9" s="4">
-        <v>0.32</v>
-      </c>
-      <c r="O9" s="4">
-        <v>3</v>
-      </c>
-      <c r="P9" s="4">
-        <v>0.96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>73</v>
-      </c>
       <c r="C10" s="3" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>27</v>
@@ -1758,7 +1687,7 @@
         <v>29</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>31</v>
@@ -1767,87 +1696,79 @@
         <v>20</v>
       </c>
       <c r="J10" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="N10" s="4">
+        <v>8.5999999999999993E-2</v>
+      </c>
+      <c r="O10" s="4">
+        <v>8</v>
+      </c>
+      <c r="P10" s="4">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
+      <c r="H11" s="4"/>
+      <c r="I11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="J11" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="N10" s="4">
-        <v>0.17</v>
-      </c>
-      <c r="O10" s="4">
+      <c r="K11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="N11" s="4">
+        <v>0.16</v>
+      </c>
+      <c r="O11" s="4">
         <v>1</v>
       </c>
-      <c r="P10" s="4">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="N11" s="4">
-        <v>8.5999999999999993E-2</v>
-      </c>
-      <c r="O11" s="4">
-        <v>8</v>
-      </c>
       <c r="P11" s="4">
-        <v>0.86</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>82</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>28</v>
@@ -1856,40 +1777,40 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="3" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="N12" s="4">
-        <v>0.16</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O12" s="4">
         <v>1</v>
       </c>
       <c r="P12" s="4">
-        <v>0.16</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="3" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>28</v>
@@ -1898,19 +1819,19 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="3" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="N13" s="4">
         <v>0.14000000000000001</v>
@@ -1924,14 +1845,14 @@
     </row>
     <row r="14" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>28</v>
@@ -1940,174 +1861,184 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="3" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="N14" s="4">
         <v>0.14000000000000001</v>
       </c>
       <c r="O14" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="P14" s="4">
-        <v>0.14000000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="120" x14ac:dyDescent="0.25">
+        <v>1.1200000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="D15" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B15" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="E15" s="4"/>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="3" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="K15" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="L15" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M15" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="L15" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M15" s="3" t="s">
+      <c r="N15" s="4">
+        <v>1.36</v>
+      </c>
+      <c r="O15" s="4">
+        <v>1</v>
+      </c>
+      <c r="P15" s="4">
+        <v>1.36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="N15" s="4">
-        <v>0.14000000000000001</v>
-      </c>
-      <c r="O15" s="4">
-        <v>8</v>
-      </c>
-      <c r="P15" s="4">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="105" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>102</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>103</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>105</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M16" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N16" s="4">
-        <v>2.78</v>
+        <v>8.3800000000000008</v>
       </c>
       <c r="O16" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P16" s="4">
-        <v>2.78</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>16.760000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="C17" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C17" s="4"/>
       <c r="D17" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
+        <v>110</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>111</v>
+      </c>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M17" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="N17" s="4">
+        <v>2.4E-2</v>
+      </c>
+      <c r="O17" s="4">
+        <v>4</v>
+      </c>
+      <c r="P17" s="4">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="E18" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>111</v>
       </c>
-      <c r="K17" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M17" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="N17" s="4">
-        <v>0.74</v>
-      </c>
-      <c r="O17" s="4">
-        <v>1</v>
-      </c>
-      <c r="P17" s="4">
-        <v>0.74</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="3" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>69</v>
+        <v>113</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>118</v>
@@ -2119,13 +2050,13 @@
         <v>119</v>
       </c>
       <c r="N18" s="4">
-        <v>1.36</v>
+        <v>0.1</v>
       </c>
       <c r="O18" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P18" s="4">
-        <v>1.36</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
@@ -2135,710 +2066,716 @@
       <c r="B19" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C19" s="4"/>
+      <c r="C19" s="3" t="s">
+        <v>120</v>
+      </c>
       <c r="D19" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
+        <v>110</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>111</v>
+      </c>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="J19" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K19" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="L19" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M19" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="J19" s="3" t="s">
+      <c r="N19" s="4">
+        <v>2.4E-2</v>
+      </c>
+      <c r="O19" s="4">
+        <v>9</v>
+      </c>
+      <c r="P19" s="4">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A20" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="B20" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="L19" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M19" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="N19" s="4">
-        <v>8.3800000000000008</v>
-      </c>
-      <c r="O19" s="4">
-        <v>2</v>
-      </c>
-      <c r="P19" s="4">
-        <v>16.760000000000002</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>128</v>
-      </c>
       <c r="C20" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>131</v>
+        <v>113</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="L20" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="N20" s="4">
-        <v>2.4E-2</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="O20" s="4">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="P20" s="4">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="J21" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="K21" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="J21" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="K21" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="L21" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="N21" s="4">
-        <v>0.1</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="O21" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P21" s="4">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J22" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="L22" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M22" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="K22" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="L22" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M22" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="N22" s="4">
-        <v>2.4E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O22" s="4">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="P22" s="4">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="N23" s="4">
-        <v>0.14399999999999999</v>
+        <v>0.1</v>
       </c>
       <c r="O23" s="4">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="P23" s="4">
-        <v>1.44</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="N24" s="4">
-        <v>1.7000000000000001E-2</v>
+        <v>0.17</v>
       </c>
       <c r="O24" s="4">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="P24" s="4">
-        <v>0.187</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>151</v>
+        <v>124</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>151</v>
+        <v>124</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="N25" s="4">
-        <v>0.1</v>
+        <v>0.60299999999999998</v>
       </c>
       <c r="O25" s="4">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="P25" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>7.24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>146</v>
+      </c>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="3" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="N26" s="4">
-        <v>0.1</v>
+        <v>0.77</v>
       </c>
       <c r="O26" s="4">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="P26" s="4">
-        <v>0.2</v>
+        <v>6.16</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="N27" s="4">
-        <v>0.17</v>
+        <v>0.1</v>
       </c>
       <c r="O27" s="4">
         <v>1</v>
       </c>
       <c r="P27" s="4">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
+        <v>161</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>111</v>
+      </c>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J28" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="K28" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="N28" s="4">
+        <v>0.22</v>
+      </c>
+      <c r="O28" s="4">
+        <v>1</v>
+      </c>
+      <c r="P28" s="4">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B29" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="J28" s="3" t="s">
+      <c r="C29" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="D29" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="E29" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F29" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="K28" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="L28" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M28" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="N28" s="4">
-        <v>0.60299999999999998</v>
-      </c>
-      <c r="O28" s="4">
-        <v>12</v>
-      </c>
-      <c r="P28" s="4">
-        <v>7.24</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="E29" s="4"/>
-      <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="3" t="s">
-        <v>166</v>
+        <v>112</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K29" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="L29" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M29" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="N29" s="4">
+        <v>0.26</v>
+      </c>
+      <c r="O29" s="4">
+        <v>16</v>
+      </c>
+      <c r="P29" s="4">
+        <v>4.16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+      <c r="A30" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="L29" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M29" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="N29" s="4">
-        <v>0.77</v>
-      </c>
-      <c r="O29" s="4">
-        <v>8</v>
-      </c>
-      <c r="P29" s="4">
-        <v>6.16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>175</v>
-      </c>
       <c r="C30" s="3" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>129</v>
+        <v>167</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
       <c r="I30" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>136</v>
+        <v>168</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="N30" s="4">
-        <v>0.1</v>
+        <v>0.26</v>
       </c>
       <c r="O30" s="4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="P30" s="4">
-        <v>0.1</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>178</v>
+        <v>151</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>178</v>
+        <v>151</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>180</v>
+        <v>110</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="3" t="s">
-        <v>20</v>
+        <v>112</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>181</v>
+        <v>113</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="N31" s="4">
-        <v>0.22</v>
+        <v>0.1</v>
       </c>
       <c r="O31" s="4">
         <v>1</v>
       </c>
       <c r="P31" s="4">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>186</v>
+        <v>111</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="I32" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>187</v>
+        <v>113</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
       <c r="N32" s="4">
-        <v>0.26</v>
+        <v>0.1</v>
       </c>
       <c r="O32" s="4">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="P32" s="4">
-        <v>4.16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>107</v>
+        <v>184</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>186</v>
+        <v>167</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="3" t="s">
-        <v>130</v>
+        <v>20</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="N33" s="4">
-        <v>0.26</v>
+        <v>0.41</v>
       </c>
       <c r="O33" s="4">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="P33" s="4">
-        <v>4.16</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>129</v>
+        <v>111</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="3" t="s">
-        <v>130</v>
+        <v>112</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>136</v>
+        <v>113</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="L34" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="N34" s="4">
         <v>0.1</v>
@@ -2852,122 +2789,106 @@
     </row>
     <row r="35" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>197</v>
-      </c>
+        <v>192</v>
+      </c>
+      <c r="C35" s="4"/>
       <c r="D35" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F35" s="3" t="s">
-        <v>129</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="3" t="s">
-        <v>130</v>
+        <v>193</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>136</v>
+        <v>194</v>
       </c>
       <c r="K35" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M35" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="N35" s="4">
+        <v>3.98</v>
+      </c>
+      <c r="O35" s="4">
+        <v>2</v>
+      </c>
+      <c r="P35" s="4">
+        <v>7.96</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>197</v>
+      </c>
+      <c r="B36" s="3" t="s">
+        <v>198</v>
+      </c>
+      <c r="C36" s="4"/>
+      <c r="D36" s="3" t="s">
         <v>199</v>
       </c>
-      <c r="L35" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M35" s="3" t="s">
+      <c r="E36" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="N35" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="O35" s="4">
-        <v>1</v>
-      </c>
-      <c r="P35" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A36" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>202</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>186</v>
-      </c>
+      <c r="F36" s="4"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="3" t="s">
-        <v>20</v>
+        <v>201</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="K36" s="3" t="s">
+        <v>202</v>
+      </c>
+      <c r="L36" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M36" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="N36" s="4">
+        <v>7.33</v>
+      </c>
+      <c r="O36" s="4">
+        <v>2</v>
+      </c>
+      <c r="P36" s="4">
+        <v>14.66</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A37" s="3" t="s">
         <v>204</v>
       </c>
-      <c r="L36" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M36" s="3" t="s">
+      <c r="B37" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="N36" s="4">
-        <v>0.41</v>
-      </c>
-      <c r="O36" s="4">
-        <v>8</v>
-      </c>
-      <c r="P36" s="4">
-        <v>4.0999999999999996</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" s="3" t="s">
+      <c r="C37" s="4"/>
+      <c r="D37" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="B37" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="C37" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F37" s="3" t="s">
-        <v>129</v>
-      </c>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="3" t="s">
-        <v>130</v>
+        <v>207</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>136</v>
+        <v>194</v>
       </c>
       <c r="K37" s="3" t="s">
         <v>208</v>
@@ -2979,16 +2900,16 @@
         <v>209</v>
       </c>
       <c r="N37" s="4">
-        <v>0.1</v>
+        <v>3.83</v>
       </c>
       <c r="O37" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="P37" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>30.64</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>210</v>
       </c>
@@ -2997,7 +2918,7 @@
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
@@ -3007,89 +2928,87 @@
         <v>212</v>
       </c>
       <c r="J38" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="K38" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="K38" s="3" t="s">
+      <c r="L38" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M38" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="L38" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M38" s="3" t="s">
+      <c r="N38" s="4">
+        <v>124.86</v>
+      </c>
+      <c r="O38" s="4">
+        <v>1</v>
+      </c>
+      <c r="P38" s="4">
+        <v>124.86</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>215</v>
       </c>
-      <c r="N38" s="4">
-        <v>3.98</v>
-      </c>
-      <c r="O38" s="4">
-        <v>2</v>
-      </c>
-      <c r="P38" s="4">
-        <v>7.96</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
+      <c r="B39" s="3" t="s">
         <v>216</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>217</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="E39" s="3" t="s">
-        <v>219</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
       <c r="I39" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="J39" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K39" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="J39" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="K39" s="3" t="s">
+      <c r="L39" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M39" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="L39" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M39" s="3" t="s">
+      <c r="N39" s="4">
+        <v>0.32</v>
+      </c>
+      <c r="O39" s="4">
+        <v>8</v>
+      </c>
+      <c r="P39" s="4">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="N39" s="4">
-        <v>7.33</v>
-      </c>
-      <c r="O39" s="4">
-        <v>2</v>
-      </c>
-      <c r="P39" s="4">
-        <v>14.66</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
+      <c r="B40" s="3" t="s">
         <v>223</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>224</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="J40" s="3" t="s">
         <v>226</v>
-      </c>
-      <c r="J40" s="3" t="s">
-        <v>213</v>
       </c>
       <c r="K40" s="3" t="s">
         <v>227</v>
@@ -3101,13 +3020,13 @@
         <v>228</v>
       </c>
       <c r="N40" s="4">
-        <v>3.83</v>
+        <v>7</v>
       </c>
       <c r="O40" s="4">
         <v>8</v>
       </c>
       <c r="P40" s="4">
-        <v>30.64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="45" x14ac:dyDescent="0.25">
@@ -3119,97 +3038,93 @@
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="3" t="s">
-        <v>107</v>
+        <v>231</v>
       </c>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
       <c r="I41" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="L41" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="N41" s="4">
-        <v>124.86</v>
+        <v>0.53</v>
       </c>
       <c r="O41" s="4">
         <v>1</v>
       </c>
       <c r="P41" s="4">
-        <v>124.86</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="3" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K42" s="3" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="L42" s="3" t="s">
-        <v>23</v>
+        <v>240</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>240</v>
-      </c>
-      <c r="N42" s="4">
-        <v>0.32</v>
-      </c>
+        <v>241</v>
+      </c>
+      <c r="N42" s="4"/>
       <c r="O42" s="4">
-        <v>8</v>
-      </c>
-      <c r="P42" s="4">
-        <v>2.56</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="P42" s="4"/>
+    </row>
+    <row r="43" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>245</v>
+        <v>194</v>
       </c>
       <c r="K43" s="3" t="s">
         <v>246</v>
@@ -3221,16 +3136,16 @@
         <v>247</v>
       </c>
       <c r="N43" s="4">
-        <v>7</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="O43" s="4">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="P43" s="4">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="75" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>248</v>
       </c>
@@ -3249,230 +3164,72 @@
         <v>251</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>213</v>
+        <v>194</v>
       </c>
       <c r="K44" s="3" t="s">
         <v>252</v>
       </c>
       <c r="L44" s="3" t="s">
-        <v>23</v>
+        <v>253</v>
       </c>
       <c r="M44" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="N44" s="4">
-        <v>0.53</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="O44" s="4">
         <v>1</v>
       </c>
       <c r="P44" s="4">
-        <v>0.53</v>
+        <v>0.56000000000000005</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B45" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="C45" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="C45" s="4"/>
       <c r="D45" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>259</v>
+        <v>23</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="N45" s="4"/>
+        <v>261</v>
+      </c>
+      <c r="N45" s="4">
+        <v>1.41</v>
+      </c>
       <c r="O45" s="4">
         <v>1</v>
       </c>
-      <c r="P45" s="4"/>
-    </row>
-    <row r="46" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A46" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="C46" s="4"/>
-      <c r="D46" s="3" t="s">
-        <v>263</v>
-      </c>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="3" t="s">
-        <v>264</v>
-      </c>
-      <c r="J46" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="K46" s="3" t="s">
-        <v>265</v>
-      </c>
-      <c r="L46" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M46" s="3" t="s">
-        <v>266</v>
-      </c>
-      <c r="N46" s="4">
-        <v>2.4300000000000002</v>
-      </c>
-      <c r="O46" s="4">
-        <v>1</v>
-      </c>
-      <c r="P46" s="4">
-        <v>2.4300000000000002</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="B47" s="3" t="s">
-        <v>268</v>
-      </c>
-      <c r="C47" s="4"/>
-      <c r="D47" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="E47" s="4"/>
-      <c r="F47" s="4"/>
-      <c r="G47" s="4"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="3" t="s">
-        <v>270</v>
-      </c>
-      <c r="J47" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="K47" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="L47" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="M47" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="N47" s="4">
-        <v>0.56000000000000005</v>
-      </c>
-      <c r="O47" s="4">
-        <v>1</v>
-      </c>
-      <c r="P47" s="4">
-        <v>0.56000000000000005</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A48" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="B48" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="C48" s="3" t="s">
-        <v>274</v>
-      </c>
-      <c r="D48" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="E48" s="4"/>
-      <c r="F48" s="4"/>
-      <c r="G48" s="4"/>
-      <c r="H48" s="4"/>
-      <c r="I48" s="3" t="s">
-        <v>277</v>
-      </c>
-      <c r="J48" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="K48" s="3" t="s">
-        <v>279</v>
-      </c>
-      <c r="L48" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M48" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="N48" s="4">
+      <c r="P45" s="4">
         <v>1.41</v>
-      </c>
-      <c r="O48" s="4">
-        <v>1</v>
-      </c>
-      <c r="P48" s="4">
-        <v>1.41</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A49" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="B49" s="3" t="s">
-        <v>282</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>283</v>
-      </c>
-      <c r="E49" s="4"/>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
-      <c r="H49" s="4"/>
-      <c r="I49" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="J49" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="K49" s="3" t="s">
-        <v>284</v>
-      </c>
-      <c r="L49" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M49" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="N49" s="4">
-        <v>3.64</v>
-      </c>
-      <c r="O49" s="4">
-        <v>1</v>
-      </c>
-      <c r="P49" s="4">
-        <v>3.64</v>
       </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="19" orientation="landscape" horizontalDpi="4294967292" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="21" orientation="landscape" horizontalDpi="4294967292" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated value 15uH instead 15mH in power supply. Added Through hole components in SMD_assembly Regenerate fabrication outputs
</commit_message>
<xml_diff>
--- a/Project Outputs for UltraZohm_Analog_ADS5272/BOM/BOM_UltraZohm_Analog_ADS5272_3v01.xlsx
+++ b/Project Outputs for UltraZohm_Analog_ADS5272/BOM/BOM_UltraZohm_Analog_ADS5272_3v01.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\UltraZohm\UZ_A_ADS5272\Project Outputs for UltraZohm_Analog_ADS5272\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\Documents\Altium_projects\UltraZohm\UZ_A_ADS5272\Project Outputs for UltraZohm_Analog_ADS5272\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{870F30B5-A0FE-43EF-BC63-1830E0C34554}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9BC76F4A-AD78-4EC9-AD84-50B4734C04B7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2940" yWindow="2460" windowWidth="14670" windowHeight="8325" xr2:uid="{43EB9E44-8CEF-4548-86FA-A424F98C0A85}"/>
+    <workbookView xWindow="1020" yWindow="1290" windowWidth="21600" windowHeight="11505" xr2:uid="{55256E5C-DE01-4CAB-9E89-2385DDB955B0}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_UltraZohm_Analog_ADS5272_3v" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="278">
   <si>
     <t>Name</t>
   </si>
@@ -216,6 +216,27 @@
     <t>732-7766-1-ND</t>
   </si>
   <si>
+    <t>68µF</t>
+  </si>
+  <si>
+    <t>C60, C61</t>
+  </si>
+  <si>
+    <t>WCAP-ATG8 THT Aluminum Electrolytic Capacitors, D6.3mm x L11mm, 68uF, +/-20%, 35VDC</t>
+  </si>
+  <si>
+    <t>+/-20%</t>
+  </si>
+  <si>
+    <t>WCAP-ATG8_6.3x11</t>
+  </si>
+  <si>
+    <t>860010573006</t>
+  </si>
+  <si>
+    <t>732-8736-1-ND</t>
+  </si>
+  <si>
     <t>10µF</t>
   </si>
   <si>
@@ -324,7 +345,40 @@
     <t>732-4981-1-ND</t>
   </si>
   <si>
-    <t>15mH</t>
+    <t>RJHSE-5380-02</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>Modular Jack WR-MJ, Tab Up, Shielded, Dual Port, Righ Angle, THT, 8P8C</t>
+  </si>
+  <si>
+    <t>Amphenol ICC</t>
+  </si>
+  <si>
+    <t>RJHSE-5380-02-ND</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>JTAG CPLD</t>
+  </si>
+  <si>
+    <t>Header, 5-Pin, Dual row, Vertical</t>
+  </si>
+  <si>
+    <t>HEADER_JTAG - MAXII Horizontal</t>
+  </si>
+  <si>
+    <t>61201021721</t>
+  </si>
+  <si>
+    <t>732-2098-ND</t>
+  </si>
+  <si>
+    <t>15uH</t>
   </si>
   <si>
     <t>L2</t>
@@ -336,7 +390,7 @@
     <t>SMT_inductor_1050_Performance</t>
   </si>
   <si>
-    <t>48150SC</t>
+    <t>Digikey</t>
   </si>
   <si>
     <t>811-3837-1-ND</t>
@@ -369,9 +423,6 @@
     <t>R1, R2, R21, R22</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>1%</t>
   </si>
   <si>
@@ -757,9 +808,6 @@
   </si>
   <si>
     <t>Intel Altera</t>
-  </si>
-  <si>
-    <t>Digikey</t>
   </si>
   <si>
     <t>544-2839-ND</t>
@@ -1204,11 +1252,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2344F444-6119-4E31-8C7D-B0DBEF4FE766}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BD2E34C-A17F-46DE-A828-2A467D6AE52C}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.5703125" customWidth="1"/>
@@ -1567,7 +1615,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="135" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>59</v>
       </c>
@@ -1578,54 +1626,50 @@
         <v>59</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>19</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="E8" s="4"/>
       <c r="F8" s="3" t="s">
-        <v>29</v>
+        <v>62</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>31</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="H8" s="4"/>
       <c r="I8" s="3" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="L8" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N8" s="4">
-        <v>0.34</v>
+        <v>0.13</v>
       </c>
       <c r="O8" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P8" s="4">
-        <v>1.02</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C9" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>65</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>27</v>
@@ -1637,7 +1681,7 @@
         <v>29</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>31</v>
@@ -1646,36 +1690,36 @@
         <v>20</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N9" s="4">
-        <v>0.17</v>
+        <v>0.34</v>
       </c>
       <c r="O9" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P9" s="4">
-        <v>0.17</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>25</v>
+        <v>72</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>27</v>
@@ -1687,7 +1731,7 @@
         <v>29</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>31</v>
@@ -1696,79 +1740,87 @@
         <v>20</v>
       </c>
       <c r="J10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="N10" s="4">
+        <v>0.17</v>
+      </c>
+      <c r="O10" s="4">
+        <v>1</v>
+      </c>
+      <c r="P10" s="4">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="J11" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="K10" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="N10" s="4">
+      <c r="K11" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="L11" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="N11" s="4">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="O10" s="4">
+      <c r="O11" s="4">
         <v>8</v>
       </c>
-      <c r="P10" s="4">
+      <c r="P11" s="4">
         <v>0.86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="120" x14ac:dyDescent="0.25">
-      <c r="A11" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="C11" s="4"/>
-      <c r="D11" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="J11" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="K11" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="L11" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M11" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="N11" s="4">
-        <v>0.16</v>
-      </c>
-      <c r="O11" s="4">
-        <v>1</v>
-      </c>
-      <c r="P11" s="4">
-        <v>0.16</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C12" s="4"/>
       <c r="D12" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E12" s="3" t="s">
         <v>28</v>
@@ -1777,40 +1829,40 @@
       <c r="G12" s="4"/>
       <c r="H12" s="4"/>
       <c r="I12" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M12" s="3" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="N12" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="O12" s="4">
         <v>1</v>
       </c>
       <c r="P12" s="4">
-        <v>0.14000000000000001</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C13" s="4"/>
       <c r="D13" s="3" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="E13" s="3" t="s">
         <v>28</v>
@@ -1819,19 +1871,19 @@
       <c r="G13" s="4"/>
       <c r="H13" s="4"/>
       <c r="I13" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="L13" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M13" s="3" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N13" s="4">
         <v>0.14000000000000001</v>
@@ -1845,14 +1897,14 @@
     </row>
     <row r="14" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C14" s="4"/>
       <c r="D14" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="E14" s="3" t="s">
         <v>28</v>
@@ -1861,921 +1913,897 @@
       <c r="G14" s="4"/>
       <c r="H14" s="4"/>
       <c r="I14" s="3" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>21</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M14" s="3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="N14" s="4">
         <v>0.14000000000000001</v>
       </c>
       <c r="O14" s="4">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="P14" s="4">
-        <v>1.1200000000000001</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>0.14000000000000001</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="120" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>95</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="C15" s="4"/>
       <c r="D15" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="E15" s="4"/>
+        <v>99</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>28</v>
+      </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
       <c r="H15" s="4"/>
       <c r="I15" s="3" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M15" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="N15" s="4">
-        <v>1.36</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O15" s="4">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="P15" s="4">
-        <v>1.36</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>1.1200000000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="105" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C16" s="4"/>
       <c r="D16" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4"/>
       <c r="G16" s="4"/>
       <c r="H16" s="4"/>
       <c r="I16" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>105</v>
       </c>
       <c r="K16" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M16" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="L16" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M16" s="3" t="s">
+      <c r="N16" s="4">
+        <v>2.78</v>
+      </c>
+      <c r="O16" s="4">
+        <v>1</v>
+      </c>
+      <c r="P16" s="4">
+        <v>2.78</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="N16" s="4">
-        <v>8.3800000000000008</v>
-      </c>
-      <c r="O16" s="4">
-        <v>2</v>
-      </c>
-      <c r="P16" s="4">
-        <v>16.760000000000002</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="4"/>
+      <c r="D17" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
       <c r="I17" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="L17" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M17" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="N17" s="4">
+        <v>0.59</v>
+      </c>
+      <c r="O17" s="4">
+        <v>1</v>
+      </c>
+      <c r="P17" s="4">
+        <v>0.59</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="B18" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="L17" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M17" s="3" t="s">
+      <c r="C18" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D18" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="N17" s="4">
-        <v>2.4E-2</v>
-      </c>
-      <c r="O17" s="4">
-        <v>4</v>
-      </c>
-      <c r="P17" s="4">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="K18" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
+      <c r="L18" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="M18" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="L18" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="N18" s="4">
-        <v>0.1</v>
-      </c>
+      <c r="N18" s="4"/>
       <c r="O18" s="4">
-        <v>2</v>
-      </c>
-      <c r="P18" s="4">
-        <v>0.2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="P18" s="4"/>
     </row>
     <row r="19" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="4"/>
+      <c r="D19" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>111</v>
-      </c>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
       <c r="I19" s="3" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L19" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M19" s="3" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="N19" s="4">
-        <v>2.4E-2</v>
+        <v>8.3800000000000008</v>
       </c>
       <c r="O19" s="4">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="P19" s="4">
-        <v>0.24</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>16.760000000000002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E20" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
       <c r="I20" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="L20" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M20" s="3" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="N20" s="4">
-        <v>0.14399999999999999</v>
+        <v>2.4E-2</v>
       </c>
       <c r="O20" s="4">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="P20" s="4">
-        <v>1.44</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E21" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
       <c r="I21" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M21" s="3" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="N21" s="4">
-        <v>1.7000000000000001E-2</v>
+        <v>0.1</v>
       </c>
       <c r="O21" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="P21" s="4">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E22" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
       <c r="I22" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="L22" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M22" s="3" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="N22" s="4">
-        <v>0.1</v>
+        <v>2.4E-2</v>
       </c>
       <c r="O22" s="4">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="P22" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E23" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
       <c r="I23" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="L23" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M23" s="3" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="N23" s="4">
-        <v>0.1</v>
+        <v>0.14399999999999999</v>
       </c>
       <c r="O23" s="4">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="P23" s="4">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>1.44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E24" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
       <c r="I24" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M24" s="3" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="N24" s="4">
-        <v>0.17</v>
+        <v>1.7000000000000001E-2</v>
       </c>
       <c r="O24" s="4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P24" s="4">
         <v>0.17</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
+        <v>107</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F25" s="3" t="s">
+        <v>128</v>
+      </c>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
       <c r="I25" s="3" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="L25" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M25" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="N25" s="4">
-        <v>0.60299999999999998</v>
+        <v>0.1</v>
       </c>
       <c r="O25" s="4">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="P25" s="4">
-        <v>7.24</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
+        <v>107</v>
+      </c>
+      <c r="E26" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>128</v>
+      </c>
       <c r="G26" s="4"/>
       <c r="H26" s="4"/>
       <c r="I26" s="3" t="s">
-        <v>147</v>
+        <v>129</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>148</v>
+        <v>130</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="L26" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="N26" s="4">
-        <v>0.77</v>
+        <v>0.1</v>
       </c>
       <c r="O26" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="P26" s="4">
-        <v>6.16</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E27" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G27" s="4"/>
       <c r="H27" s="4"/>
       <c r="I27" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="L27" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M27" s="3" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="N27" s="4">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="O27" s="4">
         <v>1</v>
       </c>
       <c r="P27" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.17</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="60" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>159</v>
+        <v>141</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>111</v>
-      </c>
+        <v>163</v>
+      </c>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
       <c r="G28" s="4"/>
       <c r="H28" s="4"/>
       <c r="I28" s="3" t="s">
-        <v>20</v>
+        <v>164</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="K28" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="L28" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M28" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="N28" s="4">
+        <v>0.60299999999999998</v>
+      </c>
+      <c r="O28" s="4">
+        <v>12</v>
+      </c>
+      <c r="P28" s="4">
+        <v>7.24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="L28" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M28" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="N28" s="4">
-        <v>0.22</v>
-      </c>
-      <c r="O28" s="4">
-        <v>1</v>
-      </c>
-      <c r="P28" s="4">
-        <v>0.22</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="90" x14ac:dyDescent="0.25">
-      <c r="A29" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>167</v>
-      </c>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
       <c r="G29" s="4"/>
       <c r="H29" s="4"/>
       <c r="I29" s="3" t="s">
-        <v>112</v>
+        <v>164</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L29" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M29" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="N29" s="4">
-        <v>0.26</v>
+        <v>0.77</v>
       </c>
       <c r="O29" s="4">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="P29" s="4">
-        <v>4.16</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="90" x14ac:dyDescent="0.25">
+        <v>6.16</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B30" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="C30" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>171</v>
-      </c>
       <c r="D30" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E30" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>167</v>
+        <v>128</v>
       </c>
       <c r="G30" s="4"/>
       <c r="H30" s="4"/>
       <c r="I30" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>168</v>
+        <v>130</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L30" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M30" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="N30" s="4">
-        <v>0.26</v>
+        <v>0.1</v>
       </c>
       <c r="O30" s="4">
-        <v>16</v>
+        <v>1</v>
       </c>
       <c r="P30" s="4">
-        <v>4.16</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>110</v>
+        <v>178</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
       <c r="I31" s="3" t="s">
-        <v>112</v>
+        <v>20</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>113</v>
+        <v>179</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M31" s="3" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="N31" s="4">
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="O31" s="4">
         <v>1</v>
       </c>
       <c r="P31" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E32" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>111</v>
+        <v>184</v>
       </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
       <c r="I32" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>113</v>
+        <v>185</v>
       </c>
       <c r="K32" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="L32" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M32" s="3" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="N32" s="4">
-        <v>0.1</v>
+        <v>0.26</v>
       </c>
       <c r="O32" s="4">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="P32" s="4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>4.16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="90" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="D33" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>184</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>167</v>
       </c>
       <c r="G33" s="4"/>
       <c r="H33" s="4"/>
       <c r="I33" s="3" t="s">
-        <v>20</v>
+        <v>129</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="K33" s="3" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="L33" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M33" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="N33" s="4">
-        <v>0.41</v>
+        <v>0.26</v>
       </c>
       <c r="O33" s="4">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="P33" s="4">
-        <v>4.0999999999999996</v>
+        <v>4.16</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>187</v>
+        <v>168</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E34" s="3" t="s">
         <v>28</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>111</v>
+        <v>128</v>
       </c>
       <c r="G34" s="4"/>
       <c r="H34" s="4"/>
       <c r="I34" s="3" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="K34" s="3" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="L34" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M34" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="N34" s="4">
         <v>0.1</v>
@@ -2789,66 +2817,76 @@
     </row>
     <row r="35" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="C35" s="4"/>
+        <v>196</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>195</v>
+      </c>
       <c r="D35" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="E35" s="4"/>
-      <c r="F35" s="4"/>
+        <v>107</v>
+      </c>
+      <c r="E35" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>128</v>
+      </c>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
       <c r="I35" s="3" t="s">
-        <v>193</v>
+        <v>129</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>194</v>
+        <v>130</v>
       </c>
       <c r="K35" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="L35" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M35" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="N35" s="4">
-        <v>3.98</v>
+        <v>0.1</v>
       </c>
       <c r="O35" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P35" s="4">
-        <v>7.96</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>198</v>
-      </c>
-      <c r="C36" s="4"/>
+        <v>200</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>199</v>
+      </c>
       <c r="D36" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="E36" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="F36" s="4"/>
+        <v>19</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>184</v>
+      </c>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
       <c r="I36" s="3" t="s">
-        <v>201</v>
+        <v>20</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>194</v>
+        <v>185</v>
       </c>
       <c r="K36" s="3" t="s">
         <v>202</v>
@@ -2860,107 +2898,115 @@
         <v>203</v>
       </c>
       <c r="N36" s="4">
-        <v>7.33</v>
+        <v>0.41</v>
       </c>
       <c r="O36" s="4">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="P36" s="4">
-        <v>14.66</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+        <v>4.0999999999999996</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="30" x14ac:dyDescent="0.25">
       <c r="A37" s="3" t="s">
         <v>204</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>205</v>
       </c>
-      <c r="C37" s="4"/>
+      <c r="C37" s="3" t="s">
+        <v>204</v>
+      </c>
       <c r="D37" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
+        <v>107</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>128</v>
+      </c>
       <c r="G37" s="4"/>
       <c r="H37" s="4"/>
       <c r="I37" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="J37" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="K37" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="L37" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M37" s="3" t="s">
         <v>207</v>
       </c>
-      <c r="J37" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="K37" s="3" t="s">
+      <c r="N37" s="4">
+        <v>0.1</v>
+      </c>
+      <c r="O37" s="4">
+        <v>1</v>
+      </c>
+      <c r="P37" s="4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="L37" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M37" s="3" t="s">
+      <c r="B38" s="3" t="s">
         <v>209</v>
-      </c>
-      <c r="N37" s="4">
-        <v>3.83</v>
-      </c>
-      <c r="O37" s="4">
-        <v>8</v>
-      </c>
-      <c r="P37" s="4">
-        <v>30.64</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A38" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>211</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="3" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
       <c r="G38" s="4"/>
       <c r="H38" s="4"/>
       <c r="I38" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="K38" s="3" t="s">
         <v>212</v>
       </c>
-      <c r="J38" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="K38" s="3" t="s">
+      <c r="L38" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M38" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="L38" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M38" s="3" t="s">
+      <c r="N38" s="4">
+        <v>3.98</v>
+      </c>
+      <c r="O38" s="4">
+        <v>2</v>
+      </c>
+      <c r="P38" s="4">
+        <v>7.96</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A39" s="3" t="s">
         <v>214</v>
       </c>
-      <c r="N38" s="4">
-        <v>124.86</v>
-      </c>
-      <c r="O38" s="4">
-        <v>1</v>
-      </c>
-      <c r="P38" s="4">
-        <v>124.86</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="45" x14ac:dyDescent="0.25">
-      <c r="A39" s="3" t="s">
+      <c r="B39" s="3" t="s">
         <v>215</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>216</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="E39" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="E39" s="4"/>
       <c r="F39" s="4"/>
       <c r="G39" s="4"/>
       <c r="H39" s="4"/>
@@ -2968,268 +3014,388 @@
         <v>218</v>
       </c>
       <c r="J39" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="K39" s="3" t="s">
         <v>219</v>
       </c>
-      <c r="K39" s="3" t="s">
+      <c r="L39" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M39" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="L39" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M39" s="3" t="s">
+      <c r="N39" s="4">
+        <v>7.33</v>
+      </c>
+      <c r="O39" s="4">
+        <v>2</v>
+      </c>
+      <c r="P39" s="4">
+        <v>14.66</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A40" s="3" t="s">
         <v>221</v>
       </c>
-      <c r="N39" s="4">
-        <v>0.32</v>
-      </c>
-      <c r="O39" s="4">
-        <v>8</v>
-      </c>
-      <c r="P39" s="4">
-        <v>2.56</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" ht="60" x14ac:dyDescent="0.25">
-      <c r="A40" s="3" t="s">
+      <c r="B40" s="3" t="s">
         <v>222</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>223</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
       <c r="I40" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="K40" s="3" t="s">
         <v>225</v>
       </c>
-      <c r="J40" s="3" t="s">
+      <c r="L40" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M40" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="K40" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="L40" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M40" s="3" t="s">
-        <v>228</v>
-      </c>
       <c r="N40" s="4">
-        <v>7</v>
+        <v>3.83</v>
       </c>
       <c r="O40" s="4">
         <v>8</v>
       </c>
       <c r="P40" s="4">
-        <v>56</v>
+        <v>30.64</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="3" t="s">
-        <v>231</v>
+        <v>107</v>
       </c>
       <c r="E41" s="4"/>
       <c r="F41" s="4"/>
       <c r="G41" s="4"/>
       <c r="H41" s="4"/>
       <c r="I41" s="3" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>194</v>
+        <v>211</v>
       </c>
       <c r="K41" s="3" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="L41" s="3" t="s">
         <v>23</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="N41" s="4">
-        <v>0.53</v>
+        <v>124.86</v>
       </c>
       <c r="O41" s="4">
         <v>1</v>
       </c>
       <c r="P41" s="4">
-        <v>0.53</v>
+        <v>124.86</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="3" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="E42" s="4"/>
       <c r="F42" s="4"/>
       <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="L42" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M42" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="J42" s="3" t="s">
+      <c r="N42" s="4">
+        <v>0.32</v>
+      </c>
+      <c r="O42" s="4">
+        <v>8</v>
+      </c>
+      <c r="P42" s="4">
+        <v>2.56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="60" x14ac:dyDescent="0.25">
+      <c r="A43" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="K42" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="L42" s="3" t="s">
+      <c r="B43" s="3" t="s">
         <v>240</v>
-      </c>
-      <c r="M42" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="N42" s="4"/>
-      <c r="O42" s="4">
-        <v>1</v>
-      </c>
-      <c r="P42" s="4"/>
-    </row>
-    <row r="43" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A43" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>243</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="3" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E43" s="4"/>
       <c r="F43" s="4"/>
       <c r="G43" s="4"/>
       <c r="H43" s="4"/>
       <c r="I43" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="J43" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="K43" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="L43" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M43" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="J43" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="K43" s="3" t="s">
+      <c r="N43" s="4">
+        <v>7</v>
+      </c>
+      <c r="O43" s="4">
+        <v>8</v>
+      </c>
+      <c r="P43" s="4">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A44" s="3" t="s">
         <v>246</v>
       </c>
-      <c r="L43" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="M43" s="3" t="s">
+      <c r="B44" s="3" t="s">
         <v>247</v>
-      </c>
-      <c r="N43" s="4">
-        <v>2.4300000000000002</v>
-      </c>
-      <c r="O43" s="4">
-        <v>1</v>
-      </c>
-      <c r="P43" s="4">
-        <v>2.4300000000000002</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="75" x14ac:dyDescent="0.25">
-      <c r="A44" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>249</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="3" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="E44" s="4"/>
       <c r="F44" s="4"/>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
       <c r="I44" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M44" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="J44" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="K44" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="L44" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="M44" s="3" t="s">
-        <v>254</v>
-      </c>
       <c r="N44" s="4">
-        <v>0.56000000000000005</v>
+        <v>0.53</v>
       </c>
       <c r="O44" s="4">
         <v>1</v>
       </c>
       <c r="P44" s="4">
-        <v>0.56000000000000005</v>
+        <v>0.53</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="45" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>255</v>
-      </c>
+        <v>253</v>
+      </c>
+      <c r="C45" s="4"/>
       <c r="D45" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="E45" s="4"/>
       <c r="F45" s="4"/>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
       <c r="I45" s="3" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="K45" s="3" t="s">
-        <v>260</v>
+        <v>252</v>
       </c>
       <c r="L45" s="3" t="s">
-        <v>23</v>
+        <v>117</v>
       </c>
       <c r="M45" s="3" t="s">
-        <v>261</v>
-      </c>
-      <c r="N45" s="4">
-        <v>1.41</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="N45" s="4"/>
       <c r="O45" s="4">
         <v>1</v>
       </c>
-      <c r="P45" s="4">
+      <c r="P45" s="4"/>
+    </row>
+    <row r="46" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A46" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>259</v>
+      </c>
+      <c r="C46" s="4"/>
+      <c r="D46" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="E46" s="4"/>
+      <c r="F46" s="4"/>
+      <c r="G46" s="4"/>
+      <c r="H46" s="4"/>
+      <c r="I46" s="3" t="s">
+        <v>261</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="K46" s="3" t="s">
+        <v>262</v>
+      </c>
+      <c r="L46" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M46" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="N46" s="4">
+        <v>2.4300000000000002</v>
+      </c>
+      <c r="O46" s="4">
+        <v>1</v>
+      </c>
+      <c r="P46" s="4">
+        <v>2.4300000000000002</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="75" x14ac:dyDescent="0.25">
+      <c r="A47" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="C47" s="4"/>
+      <c r="D47" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="E47" s="4"/>
+      <c r="F47" s="4"/>
+      <c r="G47" s="4"/>
+      <c r="H47" s="4"/>
+      <c r="I47" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="K47" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="L47" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="M47" s="3" t="s">
+        <v>270</v>
+      </c>
+      <c r="N47" s="4">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="O47" s="4">
+        <v>1</v>
+      </c>
+      <c r="P47" s="4">
+        <v>0.56000000000000005</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="45" x14ac:dyDescent="0.25">
+      <c r="A48" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="E48" s="4"/>
+      <c r="F48" s="4"/>
+      <c r="G48" s="4"/>
+      <c r="H48" s="4"/>
+      <c r="I48" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="J48" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="K48" s="3" t="s">
+        <v>276</v>
+      </c>
+      <c r="L48" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="M48" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="N48" s="4">
+        <v>1.41</v>
+      </c>
+      <c r="O48" s="4">
+        <v>1</v>
+      </c>
+      <c r="P48" s="4">
         <v>1.41</v>
       </c>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="21" orientation="landscape" horizontalDpi="4294967292" verticalDpi="1200" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="19" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>